<commit_message>
Making sure the SQO BLOE Function is using the correct versions of thecomponent indices funcitons
</commit_message>
<xml_diff>
--- a/SQO dry run/djg test - unchanged SQO BLOE output summary.xlsx
+++ b/SQO dry run/djg test - unchanged SQO BLOE output summary.xlsx
@@ -1560,7 +1560,7 @@
         <v>34</v>
       </c>
       <c r="I2" t="n">
-        <v>0.232449482790632</v>
+        <v>0.2326069101505</v>
       </c>
       <c r="J2" t="s">
         <v>15</v>
@@ -1598,7 +1598,7 @@
         <v>34</v>
       </c>
       <c r="I3" t="n">
-        <v>0.608634239976451</v>
+        <v>0.60907503658408</v>
       </c>
       <c r="J3" t="s">
         <v>31</v>
@@ -1674,7 +1674,7 @@
         <v>34</v>
       </c>
       <c r="I5" t="n">
-        <v>0.909121746711344</v>
+        <v>0.909247688599238</v>
       </c>
       <c r="J5" t="s">
         <v>31</v>
@@ -1750,7 +1750,7 @@
         <v>34</v>
       </c>
       <c r="I7" t="n">
-        <v>0.655754981373927</v>
+        <v>0.655849437789848</v>
       </c>
       <c r="J7" t="s">
         <v>31</v>

</xml_diff>

<commit_message>
re-running the sqo code with the v2.0 of the script
</commit_message>
<xml_diff>
--- a/SQO dry run/djg test - unchanged SQO BLOE output summary.xlsx
+++ b/SQO dry run/djg test - unchanged SQO BLOE output summary.xlsx
@@ -944,7 +944,7 @@
         <v>29</v>
       </c>
       <c r="I2" t="n">
-        <v>115.688285349642</v>
+        <v>110.938754784791</v>
       </c>
       <c r="J2" t="s">
         <v>30</v>
@@ -980,7 +980,7 @@
         <v>29</v>
       </c>
       <c r="I3" t="n">
-        <v>-7.16590507164652</v>
+        <v>-4.20166286851641</v>
       </c>
       <c r="J3" t="s">
         <v>31</v>
@@ -1016,7 +1016,7 @@
         <v>29</v>
       </c>
       <c r="I4" t="n">
-        <v>12.0652068770094</v>
+        <v>30.6321684845143</v>
       </c>
       <c r="J4" t="s">
         <v>31</v>
@@ -1052,7 +1052,7 @@
         <v>29</v>
       </c>
       <c r="I5" t="n">
-        <v>13.366389023643</v>
+        <v>17.1848537620817</v>
       </c>
       <c r="J5" t="s">
         <v>31</v>
@@ -1088,7 +1088,7 @@
         <v>29</v>
       </c>
       <c r="I6" t="n">
-        <v>15.0431677569128</v>
+        <v>18.6726129655443</v>
       </c>
       <c r="J6" t="s">
         <v>31</v>
@@ -1124,7 +1124,7 @@
         <v>29</v>
       </c>
       <c r="I7" t="n">
-        <v>18.9243034553919</v>
+        <v>19.8998805552463</v>
       </c>
       <c r="J7" t="s">
         <v>31</v>
@@ -1160,7 +1160,7 @@
         <v>29</v>
       </c>
       <c r="I8" t="n">
-        <v>16.2499481893049</v>
+        <v>17.1578706626853</v>
       </c>
       <c r="J8" t="s">
         <v>31</v>

</xml_diff>

<commit_message>
recalculating SQO scores from example datasets using the new v2.0 calculator
</commit_message>
<xml_diff>
--- a/SQO dry run/djg test - unchanged SQO BLOE output summary.xlsx
+++ b/SQO dry run/djg test - unchanged SQO BLOE output summary.xlsx
@@ -13,12 +13,13 @@
     <sheet name="rivpacs" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="sqo_bloe_w_mambi" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="mambi" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="potential_mismatches" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
   <si>
     <t xml:space="preserve">stationid</t>
   </si>
@@ -183,6 +184,12 @@
   </si>
   <si>
     <t xml:space="preserve">Check sample - M-AMBI ok, but limited taxa coverage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">not_on_LU_list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">did_you_mean</t>
   </si>
 </sst>
 </file>
@@ -2999,4 +3006,29 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>